<commit_message>
Redesign db_perlengkapan to match actual Excel format (TIPE/NOSIN/ACEH/RIAU/KEPRI/Type)
- Migration: new columns tipe, nosin, aceh, riau, kepri, type (drop old kode/nama/satuan/qty/keterangan)
- Alter migration added for existing installs
- Model, controller colMap/searchCols, blade headers, JS renderRow/fields all updated
- Updated perlengkapan Excel template with new column headers
</commit_message>
<xml_diff>
--- a/public/templates/template-perlengkapan.xlsx
+++ b/public/templates/template-perlengkapan.xlsx
@@ -8,33 +8,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>Kode</t>
+    <t>TIPE</t>
   </si>
   <si>
-    <t>Nama</t>
+    <t>NOSIN</t>
   </si>
   <si>
-    <t>Satuan</t>
+    <t>ACEH</t>
   </si>
   <si>
-    <t>Qty</t>
+    <t>RIAU</t>
   </si>
   <si>
-    <t>Keterangan</t>
+    <t>KEPRI</t>
   </si>
   <si>
-    <t>PK001</t>
-  </si>
-  <si>
-    <t>Helm</t>
-  </si>
-  <si>
-    <t>PCS</t>
-  </si>
-  <si>
-    <t>Perlengkapan safety</t>
+    <t>Type</t>
   </si>
 </sst>
 </file>
@@ -58,22 +49,8 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="F1" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>